<commit_message>
fix(import-grade) : excel parser
</commit_message>
<xml_diff>
--- a/src/test/resources/mock/test-update-grade.xlsx
+++ b/src/test/resources/mock/test-update-grade.xlsx
@@ -592,7 +592,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" ht="14.25">
@@ -600,7 +600,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" ht="14.25">

</xml_diff>